<commit_message>
refactor(data): Этап A унификации format_id под канон SOLO/STANDARD/PREMIUM
Баги 1-4 из DIAGNOSTICS_REPORT закрыты для 10 ниш: BARBER, DENTAL, PVZ,
PHARMACY, REPAIR_PHONE, BROW, LASH, SUGARING, MANICURE, GROCERY.

Канон: format_id = NICHE_{SOLO|STANDARD|PREMIUM} + семантические
суффиксы (HOME, MOBILE, KIOSK) для спецслучаев.

Per-niche xlsx и 08_niche_formats.xlsx теперь синхронизированы по
этим нишам — движок находит данные, расчёты возвращают корректные
цифры вместо нулей.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kz/08_niche_formats.xlsx
+++ b/data/kz/08_niche_formats.xlsx
@@ -471,6 +471,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -555,7 +556,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -680,7 +680,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -776,7 +775,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NAIL_HOME</t>
+          <t>MANICURE_HOME</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -805,7 +804,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -815,7 +813,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NAIL_SOLO</t>
+          <t>MANICURE_SOLO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -844,7 +842,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -854,7 +851,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NAIL_CABINET</t>
+          <t>MANICURE_STANDARD</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -897,7 +894,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NAIL_SALON</t>
+          <t>MANICURE_PREMIUM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -969,7 +966,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1008,7 +1004,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1018,7 +1013,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BROW_CABINET</t>
+          <t>BROW_STANDARD</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1090,7 +1085,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1129,7 +1123,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1139,7 +1132,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>LASH_CABINET</t>
+          <t>LASH_STANDARD</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1182,7 +1175,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SUGAR_HOME</t>
+          <t>SUGARING_HOME</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1211,7 +1204,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1221,7 +1213,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SUGAR_SOLO</t>
+          <t>SUGARING_SOLO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1250,7 +1242,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1260,7 +1251,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SUGAR_CABINET</t>
+          <t>SUGARING_STANDARD</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1332,7 +1323,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1371,7 +1361,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1453,7 +1442,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1549,7 +1537,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DENTAL_1CH</t>
+          <t>DENTAL_SOLO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1592,7 +1580,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DENTAL_CLINIC</t>
+          <t>DENTAL_STANDARD</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1750,7 +1738,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1803,7 +1790,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>REPAIR_POINT</t>
+          <t>REPAIR_PHONE_KIOSK</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1846,7 +1833,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>REPAIR_STUDIO</t>
+          <t>REPAIR_PHONE_STANDARD</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1918,7 +1905,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2387,7 +2373,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2985,7 +2970,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3067,7 +3051,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3636,7 +3619,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PHARM_SMALL</t>
+          <t>PHARMACY_SOLO</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3679,7 +3662,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PHARM_FULL</t>
+          <t>PHARMACY_STANDARD</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3722,7 +3705,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>GROC_KIOSK</t>
+          <t>GROCERY_SOLO</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3765,7 +3748,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>GROC_STANDARD</t>
+          <t>GROCERY_STANDARD</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3808,7 +3791,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>GROC_SUPER</t>
+          <t>GROCERY_PREMIUM</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4095,7 +4078,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4306,7 +4288,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4388,7 +4369,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4642,7 +4622,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4724,7 +4703,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5064,7 +5042,6 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5404,7 +5381,6 @@
           <t>rent_in_salon</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5887,7 +5863,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>PVZ_SMALL</t>
+          <t>PVZ_SOLO</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -5930,7 +5906,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PVZ_FULL</t>
+          <t>PVZ_STANDARD</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">

</xml_diff>